<commit_message>
Fix corrupted dropdowns in the regenerated registry Excel
OOXML dataValidation formulas must not carry a leading "=" —
openpyxl writes it verbatim and Excel then reports the workbook as
corrupted and strips the validations on repair. Write the defined
name bare and regenerate the workbook (content unchanged, verified
cell-by-cell; all 22 XML parts parse clean).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -10712,28 +10712,28 @@
   </conditionalFormatting>
   <dataValidations count="8">
     <dataValidation sqref="C3:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=MOSAIC_Countries</formula1>
+      <formula1>MOSAIC_Countries</formula1>
     </dataValidation>
     <dataValidation sqref="D3:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=MOSAIC_Themes</formula1>
+      <formula1>MOSAIC_Themes</formula1>
     </dataValidation>
     <dataValidation sqref="E3:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=MOSAIC_LLs</formula1>
+      <formula1>MOSAIC_LLs</formula1>
     </dataValidation>
     <dataValidation sqref="F3:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=MOSAIC_DataTypes</formula1>
+      <formula1>MOSAIC_DataTypes</formula1>
     </dataValidation>
     <dataValidation sqref="I3:I200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=MOSAIC_Sources</formula1>
+      <formula1>MOSAIC_Sources</formula1>
     </dataValidation>
     <dataValidation sqref="K3:K200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=MOSAIC_Access</formula1>
+      <formula1>MOSAIC_Access</formula1>
     </dataValidation>
     <dataValidation sqref="P3:P200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=MOSAIC_Migration</formula1>
+      <formula1>MOSAIC_Migration</formula1>
     </dataValidation>
     <dataValidation sqref="U3:U200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>=MOSAIC_UpdFreq</formula1>
+      <formula1>MOSAIC_UpdFreq</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Register MFL-2026-083: Crop type map, Nandi county Kenya (Zhe Guo, IFPRI)
Found as one extra row in an external old copy of the registry; its
formula ID collided with 066 (SoilGrids) — assigned the next free ID,
verified against records/ and records/_pending/. living_landscape
KEN-LVB is provisional (source row left it empty; confirm with the
owner). Details in docs/RECORDS_CHANGELOG_2026-09-16.md. Excel view
regenerated (80 rows).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -20,7 +20,7 @@
     <definedName name="MOSAIC_Access">Reference!$I$2:$I$4</definedName>
     <definedName name="MOSAIC_Migration">Reference!$O$2:$O$3</definedName>
     <definedName name="MOSAIC_UpdFreq">Reference!$Q$2:$Q$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">' Registry'!$A$2:$W$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">' Registry'!$A$2:$W$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1221,7 +1221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W81"/>
+  <dimension ref="A1:W82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -8977,8 +8977,105 @@
       </c>
       <c r="W81" s="8" t="n"/>
     </row>
+    <row r="82">
+      <c r="A82" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-083</t>
+        </is>
+      </c>
+      <c r="B82" s="10" t="inlineStr">
+        <is>
+          <t>Crop type map</t>
+        </is>
+      </c>
+      <c r="C82" s="10" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D82" s="10" t="inlineStr">
+        <is>
+          <t>Ecosystem condition</t>
+        </is>
+      </c>
+      <c r="E82" s="10" t="inlineStr">
+        <is>
+          <t>KEN-LVB — Lake Victoria Basin (Kenya)</t>
+        </is>
+      </c>
+      <c r="F82" s="10" t="inlineStr">
+        <is>
+          <t>Raster</t>
+        </is>
+      </c>
+      <c r="G82" s="10" t="inlineStr">
+        <is>
+          <t>10m</t>
+        </is>
+      </c>
+      <c r="H82" s="10" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="I82" s="10" t="inlineStr">
+        <is>
+          <t>IFPRI</t>
+        </is>
+      </c>
+      <c r="J82" s="10" t="inlineStr">
+        <is>
+          <t>z.guo@cgiar.org</t>
+        </is>
+      </c>
+      <c r="K82" s="10" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="L82" s="10" t="inlineStr">
+        <is>
+          <t>CGIAR Open Access</t>
+        </is>
+      </c>
+      <c r="M82" s="10" t="inlineStr">
+        <is>
+          <t>Validated</t>
+        </is>
+      </c>
+      <c r="N82" s="10" t="n"/>
+      <c r="O82" s="10" t="inlineStr">
+        <is>
+          <t>One drive</t>
+        </is>
+      </c>
+      <c r="P82" s="10" t="n"/>
+      <c r="Q82" s="10" t="n"/>
+      <c r="R82" s="11" t="inlineStr">
+        <is>
+          <t>Major crop type maps in Nandi county, Kenya</t>
+        </is>
+      </c>
+      <c r="S82" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="T82" s="10" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="U82" s="10" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="V82" s="10" t="n"/>
+      <c r="W82" s="10" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:W81"/>
+  <autoFilter ref="A2:W82"/>
   <conditionalFormatting sqref="K3:K300">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Open"</formula>

</xml_diff>

<commit_message>
Apply Beatriz Rodríguez's answers to the Ucayali records (MFL-2026-072 to 082)
All 11 licences replace "Other (specify in notes)": CC BY 4.0 for the
MapBiomas-derived 081 and 082, a free-download statement naming RAISG
for 075, and one naming the Peruvian government sources for the other
eight. 080 now covers 2001-2024 and notes that the 2025 update at the
source is not yet included. 082 is renamed "Accumulated Burned Area
2013-2024". STAC items, the PER-PCL collection, datasets.json and the
registry Excel are regenerated. Her verbatim answers are in
docs/RECORDS_CHANGELOG_2026-09-22.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -7944,7 +7944,7 @@
       </c>
       <c r="L71" s="8" t="inlineStr">
         <is>
-          <t>Other (specify in notes)</t>
+          <t>Free download from the Peruvian government source (MINAM/GEOBOSQUES, SERNANP, INEI); no formal license stated</t>
         </is>
       </c>
       <c r="M71" s="8" t="inlineStr">
@@ -8045,7 +8045,7 @@
       </c>
       <c r="L72" s="10" t="inlineStr">
         <is>
-          <t>Other (specify in notes)</t>
+          <t>Free download from the Peruvian government source (MINAM/GEOBOSQUES, SERNANP, INEI); no formal license stated</t>
         </is>
       </c>
       <c r="M72" s="10" t="inlineStr">
@@ -8146,7 +8146,7 @@
       </c>
       <c r="L73" s="8" t="inlineStr">
         <is>
-          <t>Other (specify in notes)</t>
+          <t>Free download from the Peruvian government source (MINAM/GEOBOSQUES, SERNANP, INEI); no formal license stated</t>
         </is>
       </c>
       <c r="M73" s="8" t="inlineStr">
@@ -8247,7 +8247,7 @@
       </c>
       <c r="L74" s="10" t="inlineStr">
         <is>
-          <t>Other (specify in notes)</t>
+          <t>Free download from RAISG; no formal license stated</t>
         </is>
       </c>
       <c r="M74" s="10" t="inlineStr">
@@ -8344,7 +8344,7 @@
       </c>
       <c r="L75" s="8" t="inlineStr">
         <is>
-          <t>Other (specify in notes)</t>
+          <t>Free download from the Peruvian government source (MINAM/GEOBOSQUES, SERNANP, INEI); no formal license stated</t>
         </is>
       </c>
       <c r="M75" s="8" t="inlineStr">
@@ -8441,7 +8441,7 @@
       </c>
       <c r="L76" s="10" t="inlineStr">
         <is>
-          <t>Other (specify in notes)</t>
+          <t>Free download from the Peruvian government source (MINAM/GEOBOSQUES, SERNANP, INEI); no formal license stated</t>
         </is>
       </c>
       <c r="M76" s="10" t="inlineStr">
@@ -8538,7 +8538,7 @@
       </c>
       <c r="L77" s="8" t="inlineStr">
         <is>
-          <t>Other (specify in notes)</t>
+          <t>Free download from the Peruvian government source (MINAM/GEOBOSQUES, SERNANP, INEI); no formal license stated</t>
         </is>
       </c>
       <c r="M77" s="8" t="inlineStr">
@@ -8635,7 +8635,7 @@
       </c>
       <c r="L78" s="10" t="inlineStr">
         <is>
-          <t>Other (specify in notes)</t>
+          <t>Free download from the Peruvian government source (MINAM/GEOBOSQUES, SERNANP, INEI); no formal license stated</t>
         </is>
       </c>
       <c r="M78" s="10" t="inlineStr">
@@ -8732,7 +8732,7 @@
       </c>
       <c r="L79" s="8" t="inlineStr">
         <is>
-          <t>Other (specify in notes)</t>
+          <t>Free download from the Peruvian government source (MINAM/GEOBOSQUES, SERNANP, INEI); no formal license stated</t>
         </is>
       </c>
       <c r="M79" s="8" t="inlineStr">
@@ -8750,7 +8750,7 @@
       <c r="Q79" s="8" t="n"/>
       <c r="R79" s="9" t="inlineStr">
         <is>
-          <t>Annual forest loss from 2001-2025 in Ucayali, derived from MINAM’s GEOBOSQUES forest monitoring dataset and spatially aggregated by provinces and districts</t>
+          <t>Annual forest loss from 2001-2024 in Ucayali, derived from MINAM’s GEOBOSQUES forest monitoring dataset and spatially aggregated by provinces and districts. The 2025 update published at source is not yet included in this layer.</t>
         </is>
       </c>
       <c r="S79" s="8" t="inlineStr">
@@ -8833,7 +8833,7 @@
       </c>
       <c r="L80" s="10" t="inlineStr">
         <is>
-          <t>Other (specify in notes)</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
       <c r="M80" s="10" t="inlineStr">
@@ -8884,7 +8884,7 @@
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>Annual Burned Area</t>
+          <t>Accumulated Burned Area 2013-2024</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
@@ -8934,7 +8934,7 @@
       </c>
       <c r="L81" s="8" t="inlineStr">
         <is>
-          <t>Other (specify in notes)</t>
+          <t>CC BY 4.0</t>
         </is>
       </c>
       <c r="M81" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Clear text typed into date_registered on 040, 041, 050 and 051
"Drive" (040, 041) and "MRC produced the data" (050, 051) were copies of
current_location and description; the real registration dates are
unknown, so the field is null. Registry Excel regenerated; STAC and
datasets.json unchanged. Details: docs/RECORDS_CHANGELOG_2026-09-29.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -5180,11 +5180,7 @@
           <t>Agroecological zonations</t>
         </is>
       </c>
-      <c r="S42" s="10" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
+      <c r="S42" s="10" t="n"/>
       <c r="T42" s="10" t="n"/>
       <c r="U42" s="10" t="n"/>
       <c r="V42" s="10" t="inlineStr">
@@ -5269,11 +5265,7 @@
           <t>Agroecological zonations</t>
         </is>
       </c>
-      <c r="S43" s="8" t="inlineStr">
-        <is>
-          <t>Drive</t>
-        </is>
-      </c>
+      <c r="S43" s="8" t="n"/>
       <c r="T43" s="8" t="n"/>
       <c r="U43" s="8" t="inlineStr">
         <is>
@@ -5839,11 +5831,7 @@
           <t>MRC produced the data</t>
         </is>
       </c>
-      <c r="S49" s="8" t="inlineStr">
-        <is>
-          <t>MRC produced the data</t>
-        </is>
-      </c>
+      <c r="S49" s="8" t="n"/>
       <c r="T49" s="8" t="inlineStr">
         <is>
           <t>NA</t>
@@ -5940,11 +5928,7 @@
           <t>MRC produced the data</t>
         </is>
       </c>
-      <c r="S50" s="10" t="inlineStr">
-        <is>
-          <t>MRC produced the data</t>
-        </is>
-      </c>
+      <c r="S50" s="10" t="n"/>
       <c r="T50" s="10" t="inlineStr">
         <is>
           <t>NA</t>

</xml_diff>

<commit_message>
Register eight ILRI datasets for the Lake Victoria Basin (MFL-2026-085 to 092)
From ILRI's filled registration template (Ambica Paliwal, 2026-09-29):
Landscape Resources, Resource change, Environmental challenges, Climate
risks, Livelihood resources, Conflicts, Drivers of change and
Restoration opportunities. All are vector layers at basin level for
2026, restricted to the data owner.

Titles and descriptions are kept verbatim. The landscape, theme
spellings, licence and contact follow the catalog's vocabulary.
Access is Restricted (sent as "CGIAR internal/Restricted", to confirm)
and processing status is Raw, because the datasets are still being
processed. KEN-LVB now holds 10 records. Details and open questions:
docs/RECORDS_CHANGELOG_2026-09-30.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog/MFL_Dataset_Registry.xlsx
+++ b/catalog/MFL_Dataset_Registry.xlsx
@@ -20,7 +20,7 @@
     <definedName name="MOSAIC_Access">Reference!$I$2:$I$4</definedName>
     <definedName name="MOSAIC_Migration">Reference!$O$2:$O$3</definedName>
     <definedName name="MOSAIC_UpdFreq">Reference!$Q$2:$Q$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">' Registry'!$A$2:$W$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">' Registry'!$A$2:$W$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1221,7 +1221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W83"/>
+  <dimension ref="A1:W91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -9167,8 +9167,816 @@
       </c>
       <c r="W83" s="8" t="n"/>
     </row>
+    <row r="84">
+      <c r="A84" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-085</t>
+        </is>
+      </c>
+      <c r="B84" s="10" t="inlineStr">
+        <is>
+          <t>Landscape Resources</t>
+        </is>
+      </c>
+      <c r="C84" s="10" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D84" s="10" t="inlineStr">
+        <is>
+          <t>Ecosystem services</t>
+        </is>
+      </c>
+      <c r="E84" s="10" t="inlineStr">
+        <is>
+          <t>KEN-LVB — Lake Victoria Basin (Kenya)</t>
+        </is>
+      </c>
+      <c r="F84" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G84" s="10" t="inlineStr">
+        <is>
+          <t>Basin level</t>
+        </is>
+      </c>
+      <c r="H84" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I84" s="10" t="inlineStr">
+        <is>
+          <t>ILRI</t>
+        </is>
+      </c>
+      <c r="J84" s="10" t="inlineStr">
+        <is>
+          <t>Ambica Paliwal (a.paliwal@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K84" s="10" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="L84" s="10" t="inlineStr">
+        <is>
+          <t>Restricted — contact data owner</t>
+        </is>
+      </c>
+      <c r="M84" s="10" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N84" s="10" t="n"/>
+      <c r="O84" s="10" t="inlineStr">
+        <is>
+          <t>One drive</t>
+        </is>
+      </c>
+      <c r="P84" s="10" t="n"/>
+      <c r="Q84" s="10" t="n"/>
+      <c r="R84" s="11" t="inlineStr">
+        <is>
+          <t>Key natural resources and the ecosystem services they provide to local communities.</t>
+        </is>
+      </c>
+      <c r="S84" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T84" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U84" s="10" t="inlineStr">
+        <is>
+          <t>On-demand</t>
+        </is>
+      </c>
+      <c r="V84" s="10" t="inlineStr">
+        <is>
+          <t>Internal Available on Request</t>
+        </is>
+      </c>
+      <c r="W84" s="10" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-086</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="inlineStr">
+        <is>
+          <t>Resource change</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="inlineStr">
+        <is>
+          <t>Ecosystem condition</t>
+        </is>
+      </c>
+      <c r="E85" s="8" t="inlineStr">
+        <is>
+          <t>KEN-LVB — Lake Victoria Basin (Kenya)</t>
+        </is>
+      </c>
+      <c r="F85" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G85" s="8" t="inlineStr">
+        <is>
+          <t>Basin level</t>
+        </is>
+      </c>
+      <c r="H85" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I85" s="8" t="inlineStr">
+        <is>
+          <t>ILRI</t>
+        </is>
+      </c>
+      <c r="J85" s="8" t="inlineStr">
+        <is>
+          <t>Ambica Paliwal (a.paliwal@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K85" s="8" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="L85" s="8" t="inlineStr">
+        <is>
+          <t>Restricted — contact data owner</t>
+        </is>
+      </c>
+      <c r="M85" s="8" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N85" s="8" t="n"/>
+      <c r="O85" s="8" t="inlineStr">
+        <is>
+          <t>One drive</t>
+        </is>
+      </c>
+      <c r="P85" s="8" t="n"/>
+      <c r="Q85" s="8" t="n"/>
+      <c r="R85" s="9" t="inlineStr">
+        <is>
+          <t>Changes in the condition and availability of key resources over time.</t>
+        </is>
+      </c>
+      <c r="S85" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T85" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U85" s="8" t="inlineStr">
+        <is>
+          <t>On-demand</t>
+        </is>
+      </c>
+      <c r="V85" s="8" t="inlineStr">
+        <is>
+          <t>Internal Available on Request</t>
+        </is>
+      </c>
+      <c r="W85" s="8" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-087</t>
+        </is>
+      </c>
+      <c r="B86" s="10" t="inlineStr">
+        <is>
+          <t>Environmental challenges</t>
+        </is>
+      </c>
+      <c r="C86" s="10" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D86" s="10" t="inlineStr">
+        <is>
+          <t>Degradation / land health</t>
+        </is>
+      </c>
+      <c r="E86" s="10" t="inlineStr">
+        <is>
+          <t>KEN-LVB — Lake Victoria Basin (Kenya)</t>
+        </is>
+      </c>
+      <c r="F86" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G86" s="10" t="inlineStr">
+        <is>
+          <t>Basin level</t>
+        </is>
+      </c>
+      <c r="H86" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I86" s="10" t="inlineStr">
+        <is>
+          <t>ILRI</t>
+        </is>
+      </c>
+      <c r="J86" s="10" t="inlineStr">
+        <is>
+          <t>Ambica Paliwal (a.paliwal@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K86" s="10" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="L86" s="10" t="inlineStr">
+        <is>
+          <t>Restricted — contact data owner</t>
+        </is>
+      </c>
+      <c r="M86" s="10" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N86" s="10" t="n"/>
+      <c r="O86" s="10" t="inlineStr">
+        <is>
+          <t>One drive</t>
+        </is>
+      </c>
+      <c r="P86" s="10" t="n"/>
+      <c r="Q86" s="10" t="n"/>
+      <c r="R86" s="11" t="inlineStr">
+        <is>
+          <t>Areas affected by environmental degradation and land-health challenges.</t>
+        </is>
+      </c>
+      <c r="S86" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T86" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U86" s="10" t="inlineStr">
+        <is>
+          <t>On-demand</t>
+        </is>
+      </c>
+      <c r="V86" s="10" t="inlineStr">
+        <is>
+          <t>Internal Available on Request</t>
+        </is>
+      </c>
+      <c r="W86" s="10" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-088</t>
+        </is>
+      </c>
+      <c r="B87" s="8" t="inlineStr">
+        <is>
+          <t>Climate risks</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="inlineStr">
+        <is>
+          <t>Ecosystem condition</t>
+        </is>
+      </c>
+      <c r="E87" s="8" t="inlineStr">
+        <is>
+          <t>KEN-LVB — Lake Victoria Basin (Kenya)</t>
+        </is>
+      </c>
+      <c r="F87" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G87" s="8" t="inlineStr">
+        <is>
+          <t>Basin level</t>
+        </is>
+      </c>
+      <c r="H87" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I87" s="8" t="inlineStr">
+        <is>
+          <t>ILRI</t>
+        </is>
+      </c>
+      <c r="J87" s="8" t="inlineStr">
+        <is>
+          <t>Ambica Paliwal (a.paliwal@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K87" s="8" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="L87" s="8" t="inlineStr">
+        <is>
+          <t>Restricted — contact data owner</t>
+        </is>
+      </c>
+      <c r="M87" s="8" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N87" s="8" t="n"/>
+      <c r="O87" s="8" t="inlineStr">
+        <is>
+          <t>One drive</t>
+        </is>
+      </c>
+      <c r="P87" s="8" t="n"/>
+      <c r="Q87" s="8" t="n"/>
+      <c r="R87" s="9" t="inlineStr">
+        <is>
+          <t>Areas exposed to climate-related environmental risks and stress.</t>
+        </is>
+      </c>
+      <c r="S87" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T87" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U87" s="8" t="inlineStr">
+        <is>
+          <t>On-demand</t>
+        </is>
+      </c>
+      <c r="V87" s="8" t="inlineStr">
+        <is>
+          <t>Internal Available on Request</t>
+        </is>
+      </c>
+      <c r="W87" s="8" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-089</t>
+        </is>
+      </c>
+      <c r="B88" s="10" t="inlineStr">
+        <is>
+          <t>Livelihood resources</t>
+        </is>
+      </c>
+      <c r="C88" s="10" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D88" s="10" t="inlineStr">
+        <is>
+          <t>Socio-economic / livelihoods</t>
+        </is>
+      </c>
+      <c r="E88" s="10" t="inlineStr">
+        <is>
+          <t>KEN-LVB — Lake Victoria Basin (Kenya)</t>
+        </is>
+      </c>
+      <c r="F88" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G88" s="10" t="inlineStr">
+        <is>
+          <t>Basin level</t>
+        </is>
+      </c>
+      <c r="H88" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I88" s="10" t="inlineStr">
+        <is>
+          <t>ILRI</t>
+        </is>
+      </c>
+      <c r="J88" s="10" t="inlineStr">
+        <is>
+          <t>Ambica Paliwal (a.paliwal@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K88" s="10" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="L88" s="10" t="inlineStr">
+        <is>
+          <t>Restricted — contact data owner</t>
+        </is>
+      </c>
+      <c r="M88" s="10" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N88" s="10" t="n"/>
+      <c r="O88" s="10" t="inlineStr">
+        <is>
+          <t>One drive</t>
+        </is>
+      </c>
+      <c r="P88" s="10" t="n"/>
+      <c r="Q88" s="10" t="n"/>
+      <c r="R88" s="11" t="inlineStr">
+        <is>
+          <t>Resources and infrastructure that support local livelihoods and economic activities.</t>
+        </is>
+      </c>
+      <c r="S88" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T88" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U88" s="10" t="inlineStr">
+        <is>
+          <t>On-demand</t>
+        </is>
+      </c>
+      <c r="V88" s="10" t="inlineStr">
+        <is>
+          <t>Internal Available on Request</t>
+        </is>
+      </c>
+      <c r="W88" s="10" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-090</t>
+        </is>
+      </c>
+      <c r="B89" s="8" t="inlineStr">
+        <is>
+          <t>Conflicts</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="inlineStr">
+        <is>
+          <t>Socio-economic / livelihoods</t>
+        </is>
+      </c>
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t>KEN-LVB — Lake Victoria Basin (Kenya)</t>
+        </is>
+      </c>
+      <c r="F89" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G89" s="8" t="inlineStr">
+        <is>
+          <t>Basin level</t>
+        </is>
+      </c>
+      <c r="H89" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I89" s="8" t="inlineStr">
+        <is>
+          <t>ILRI</t>
+        </is>
+      </c>
+      <c r="J89" s="8" t="inlineStr">
+        <is>
+          <t>Ambica Paliwal (a.paliwal@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K89" s="8" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="L89" s="8" t="inlineStr">
+        <is>
+          <t>Restricted — contact data owner</t>
+        </is>
+      </c>
+      <c r="M89" s="8" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N89" s="8" t="n"/>
+      <c r="O89" s="8" t="inlineStr">
+        <is>
+          <t>One drive</t>
+        </is>
+      </c>
+      <c r="P89" s="8" t="n"/>
+      <c r="Q89" s="8" t="n"/>
+      <c r="R89" s="9" t="inlineStr">
+        <is>
+          <t>Locations and resources affected by conflicts and competing uses</t>
+        </is>
+      </c>
+      <c r="S89" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T89" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U89" s="8" t="inlineStr">
+        <is>
+          <t>On-demand</t>
+        </is>
+      </c>
+      <c r="V89" s="8" t="inlineStr">
+        <is>
+          <t>Internal Available on Request</t>
+        </is>
+      </c>
+      <c r="W89" s="8" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="10" t="inlineStr">
+        <is>
+          <t>MFL-2026-091</t>
+        </is>
+      </c>
+      <c r="B90" s="10" t="inlineStr">
+        <is>
+          <t>Drivers of change</t>
+        </is>
+      </c>
+      <c r="C90" s="10" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D90" s="10" t="inlineStr">
+        <is>
+          <t>Pressures / drivers</t>
+        </is>
+      </c>
+      <c r="E90" s="10" t="inlineStr">
+        <is>
+          <t>KEN-LVB — Lake Victoria Basin (Kenya)</t>
+        </is>
+      </c>
+      <c r="F90" s="10" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G90" s="10" t="inlineStr">
+        <is>
+          <t>Basin level</t>
+        </is>
+      </c>
+      <c r="H90" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I90" s="10" t="inlineStr">
+        <is>
+          <t>ILRI</t>
+        </is>
+      </c>
+      <c r="J90" s="10" t="inlineStr">
+        <is>
+          <t>Ambica Paliwal (a.paliwal@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K90" s="10" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="L90" s="10" t="inlineStr">
+        <is>
+          <t>Restricted — contact data owner</t>
+        </is>
+      </c>
+      <c r="M90" s="10" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N90" s="10" t="n"/>
+      <c r="O90" s="10" t="inlineStr">
+        <is>
+          <t>One drive</t>
+        </is>
+      </c>
+      <c r="P90" s="10" t="n"/>
+      <c r="Q90" s="10" t="n"/>
+      <c r="R90" s="11" t="inlineStr">
+        <is>
+          <t>Key human and environmental drivers influencing landscape change.</t>
+        </is>
+      </c>
+      <c r="S90" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T90" s="10" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U90" s="10" t="inlineStr">
+        <is>
+          <t>On-demand</t>
+        </is>
+      </c>
+      <c r="V90" s="10" t="inlineStr">
+        <is>
+          <t>Internal Available on Request</t>
+        </is>
+      </c>
+      <c r="W90" s="10" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="inlineStr">
+        <is>
+          <t>MFL-2026-092</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="inlineStr">
+        <is>
+          <t>Restoration opportunities</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr">
+        <is>
+          <t>Kenya</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="inlineStr">
+        <is>
+          <t>Decision-support outputs</t>
+        </is>
+      </c>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t>KEN-LVB — Lake Victoria Basin (Kenya)</t>
+        </is>
+      </c>
+      <c r="F91" s="8" t="inlineStr">
+        <is>
+          <t>Vector</t>
+        </is>
+      </c>
+      <c r="G91" s="8" t="inlineStr">
+        <is>
+          <t>Basin level</t>
+        </is>
+      </c>
+      <c r="H91" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="I91" s="8" t="inlineStr">
+        <is>
+          <t>ILRI</t>
+        </is>
+      </c>
+      <c r="J91" s="8" t="inlineStr">
+        <is>
+          <t>Ambica Paliwal (a.paliwal@cgiar.org)</t>
+        </is>
+      </c>
+      <c r="K91" s="8" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="L91" s="8" t="inlineStr">
+        <is>
+          <t>Restricted — contact data owner</t>
+        </is>
+      </c>
+      <c r="M91" s="8" t="inlineStr">
+        <is>
+          <t>Raw</t>
+        </is>
+      </c>
+      <c r="N91" s="8" t="n"/>
+      <c r="O91" s="8" t="inlineStr">
+        <is>
+          <t>One drive</t>
+        </is>
+      </c>
+      <c r="P91" s="8" t="n"/>
+      <c r="Q91" s="8" t="n"/>
+      <c r="R91" s="9" t="inlineStr">
+        <is>
+          <t>Priority areas and opportunities for restoration and targeted investment.</t>
+        </is>
+      </c>
+      <c r="S91" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="T91" s="8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="U91" s="8" t="inlineStr">
+        <is>
+          <t>On-demand</t>
+        </is>
+      </c>
+      <c r="V91" s="8" t="inlineStr">
+        <is>
+          <t>Internal Available on Request</t>
+        </is>
+      </c>
+      <c r="W91" s="8" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:W83"/>
+  <autoFilter ref="A2:W91"/>
   <conditionalFormatting sqref="K3:K300">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Open"</formula>

</xml_diff>